<commit_message>
Start simulation from 2007, update market data and AMPL paths for Mac
- simStartYear configurable (set to 2007, easy to change back to 2005)
- Updated FX and yield curve Excel files with extended date ranges
- forwardRates.m: Mac-compatible paths using fullfile()
- runCreateInterestRateCurves.m: 9 thesis currencies, firstDate=2007
- runPA.m/runMC.m: startDate aligned to 2007
- Still need to regenerate .mat yield curve files (requires AMPL license)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/matlabExjobb2026/marketData/allRIC.xlsx
+++ b/matlabExjobb2026/marketData/allRIC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\research\companyEarnings\matlab\marketData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liuonline-my.sharepoint.com/personal/joahu849_student_liu_se/Documents/EXJOBB Sandvik/5. Implementering/matlabExjobb2026/marketData2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{044F3FF5-A645-4B7B-93EF-AE144CAC8E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{044F3FF5-A645-4B7B-93EF-AE144CAC8E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA5EDA92-0764-4F4B-9E53-6DE0EB466CBB}"/>
   <bookViews>
-    <workbookView xWindow="810" yWindow="-120" windowWidth="28110" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>USDONZ=R;USDTNZ=R;USDSNZ=R;USD1WZ=R;USD2WZ=R;USD1MZ=R;USD2MZ=R;USD3MZ=R;USD6MZ=R;USD9MZ=R;USD1YZ=R;USD1Y3MZ=R;USD1Y6MZ=R;USD1Y9MZ=R;USD2YZ=R;USD2Y3MZ=R;USD2Y6MZ=R;USD2Y9MZ=R;USD3YZ=R;USD3Y3MZ=R;USD3Y6MZ=R;USD3Y9MZ=R;USD4YZ=R;USD4Y3MZ=R;USD4Y6MZ=R;USD4Y9MZ=R;USD5YZ=R;USD5Y3MZ=R;USD5Y6MZ=R;USD5Y9MZ=R;USD6YZ=R;USD6Y3MZ=R;USD6Y6MZ=R;USD6Y9MZ=R;USD7YZ=R;USD7Y3MZ=R;USD7Y6MZ=R;USD7Y9MZ=R;USD8YZ=R;USD8Y3MZ=R;USD8Y6MZ=R;USD8Y9MZ=R;USD9YZ=R;USD9Y3MZ=R;USD9Y6MZ=R;USD9Y9MZ=R;USD10YZ=R;USD11YZ=R;USD12YZ=R;USD13YZ=R;USD14YZ=R;USD15YZ=R;USD20YZ=R;USD25YZ=R;USD30YZ=R;USD40YZ=R;USD50YZ=R</t>
   </si>
@@ -44,73 +44,25 @@
     <t>AUDONZ=R;AUDTNZ=R;AUDSNZ=R;AUD1WZ=R;AUD2WZ=R;AUD1MZ=R;AUD2MZ=R;AUD3MZ=R;AUD6MZ=R;AUD9MZ=R;AUD1YZ=R;AUD1Y3MZ=R;AUD1Y6MZ=R;AUD1Y9MZ=R;AUD2YZ=R;AUD2Y3MZ=R;AUD2Y6MZ=R;AUD2Y9MZ=R;AUD3YZ=R;AUD3Y3MZ=R;AUD3Y6MZ=R;AUD3Y9MZ=R;AUD4YZ=R;AUD4Y3MZ=R;AUD4Y6MZ=R;AUD4Y9MZ=R;AUD5YZ=R;AUD5Y3MZ=R;AUD5Y6MZ=R;AUD5Y9MZ=R;AUD6YZ=R;AUD6Y3MZ=R;AUD6Y6MZ=R;AUD6Y9MZ=R;AUD7YZ=R;AUD7Y3MZ=R;AUD7Y6MZ=R;AUD7Y9MZ=R;AUD8YZ=R;AUD8Y3MZ=R;AUD8Y6MZ=R;AUD8Y9MZ=R;AUD9YZ=R;AUD9Y3MZ=R;AUD9Y6MZ=R;AUD9Y9MZ=R;AUD10YZ=R;AUD11YZ=R;AUD12YZ=R;AUD13YZ=R;AUD14YZ=R;AUD15YZ=R;AUD20YZ=R;AUD25YZ=R;AUD30YZ=R;AUD40YZ=R;AUD50YZ=R</t>
   </si>
   <si>
-    <t>BGNONZ=R;BGNTNZ=R;BGNSNZ=R;BGN1WZ=R;BGN2WZ=R;BGN1MZ=R;BGN2MZ=R;BGN3MZ=R;BGN6MZ=R;BGN9MZ=R;BGN1YZ=R;BGN1Y3MZ=R;BGN1Y6MZ=R;BGN1Y9MZ=R;BGN2YZ=R;BGN2Y3MZ=R;BGN2Y6MZ=R;BGN2Y9MZ=R;BGN3YZ=R;BGN3Y3MZ=R;BGN3Y6MZ=R;BGN3Y9MZ=R;BGN4YZ=R;BGN4Y3MZ=R;BGN4Y6MZ=R;BGN4Y9MZ=R;BGN5YZ=R;BGN5Y3MZ=R;BGN5Y6MZ=R;BGN5Y9MZ=R;BGN6YZ=R;BGN6Y3MZ=R;BGN6Y6MZ=R;BGN6Y9MZ=R;BGN7YZ=R;BGN7Y3MZ=R;BGN7Y6MZ=R;BGN7Y9MZ=R;BGN8YZ=R;BGN8Y3MZ=R;BGN8Y6MZ=R;BGN8Y9MZ=R;BGN9YZ=R;BGN9Y3MZ=R;BGN9Y6MZ=R;BGN9Y9MZ=R;BGN10YZ=R;BGN11YZ=R;BGN12YZ=R;BGN13YZ=R;BGN14YZ=R;BGN15YZ=R;BGN20YZ=R;BGN25YZ=R;BGN30YZ=R;BGN40YZ=R;BGN50YZ=R</t>
-  </si>
-  <si>
-    <t>BWPONZ=R;BWPTNZ=R;BWPSNZ=R;BWP1WZ=R;BWP2WZ=R;BWP1MZ=R;BWP2MZ=R;BWP3MZ=R;BWP6MZ=R;BWP9MZ=R;BWP1YZ=R;BWP1Y3MZ=R;BWP1Y6MZ=R;BWP1Y9MZ=R;BWP2YZ=R;BWP2Y3MZ=R;BWP2Y6MZ=R;BWP2Y9MZ=R;BWP3YZ=R;BWP3Y3MZ=R;BWP3Y6MZ=R;BWP3Y9MZ=R;BWP4YZ=R;BWP4Y3MZ=R;BWP4Y6MZ=R;BWP4Y9MZ=R;BWP5YZ=R;BWP5Y3MZ=R;BWP5Y6MZ=R;BWP5Y9MZ=R;BWP6YZ=R;BWP6Y3MZ=R;BWP6Y6MZ=R;BWP6Y9MZ=R;BWP7YZ=R;BWP7Y3MZ=R;BWP7Y6MZ=R;BWP7Y9MZ=R;BWP8YZ=R;BWP8Y3MZ=R;BWP8Y6MZ=R;BWP8Y9MZ=R;BWP9YZ=R;BWP9Y3MZ=R;BWP9Y6MZ=R;BWP9Y9MZ=R;BWP10YZ=R;BWP11YZ=R;BWP12YZ=R;BWP13YZ=R;BWP14YZ=R;BWP15YZ=R;BWP20YZ=R;BWP25YZ=R;BWP30YZ=R;BWP40YZ=R;BWP50YZ=R</t>
-  </si>
-  <si>
     <t>CADONZ=R;CADTNZ=R;CADSNZ=R;CAD1WZ=R;CAD2WZ=R;CAD1MZ=R;CAD2MZ=R;CAD3MZ=R;CAD6MZ=R;CAD9MZ=R;CAD1YZ=R;CAD1Y3MZ=R;CAD1Y6MZ=R;CAD1Y9MZ=R;CAD2YZ=R;CAD2Y3MZ=R;CAD2Y6MZ=R;CAD2Y9MZ=R;CAD3YZ=R;CAD3Y3MZ=R;CAD3Y6MZ=R;CAD3Y9MZ=R;CAD4YZ=R;CAD4Y3MZ=R;CAD4Y6MZ=R;CAD4Y9MZ=R;CAD5YZ=R;CAD5Y3MZ=R;CAD5Y6MZ=R;CAD5Y9MZ=R;CAD6YZ=R;CAD6Y3MZ=R;CAD6Y6MZ=R;CAD6Y9MZ=R;CAD7YZ=R;CAD7Y3MZ=R;CAD7Y6MZ=R;CAD7Y9MZ=R;CAD8YZ=R;CAD8Y3MZ=R;CAD8Y6MZ=R;CAD8Y9MZ=R;CAD9YZ=R;CAD9Y3MZ=R;CAD9Y6MZ=R;CAD9Y9MZ=R;CAD10YZ=R;CAD11YZ=R;CAD12YZ=R;CAD13YZ=R;CAD14YZ=R;CAD15YZ=R;CAD20YZ=R;CAD25YZ=R;CAD30YZ=R;CAD40YZ=R;CAD50YZ=R</t>
   </si>
   <si>
-    <t>CHFONZ=R;CHFTNZ=R;CHFSNZ=R;CHF1WZ=R;CHF2WZ=R;CHF1MZ=R;CHF2MZ=R;CHF3MZ=R;CHF6MZ=R;CHF9MZ=R;CHF1YZ=R;CHF1Y3MZ=R;CHF1Y6MZ=R;CHF1Y9MZ=R;CHF2YZ=R;CHF2Y3MZ=R;CHF2Y6MZ=R;CHF2Y9MZ=R;CHF3YZ=R;CHF3Y3MZ=R;CHF3Y6MZ=R;CHF3Y9MZ=R;CHF4YZ=R;CHF4Y3MZ=R;CHF4Y6MZ=R;CHF4Y9MZ=R;CHF5YZ=R;CHF5Y3MZ=R;CHF5Y6MZ=R;CHF5Y9MZ=R;CHF6YZ=R;CHF6Y3MZ=R;CHF6Y6MZ=R;CHF6Y9MZ=R;CHF7YZ=R;CHF7Y3MZ=R;CHF7Y6MZ=R;CHF7Y9MZ=R;CHF8YZ=R;CHF8Y3MZ=R;CHF8Y6MZ=R;CHF8Y9MZ=R;CHF9YZ=R;CHF9Y3MZ=R;CHF9Y6MZ=R;CHF9Y9MZ=R;CHF10YZ=R;CHF11YZ=R;CHF12YZ=R;CHF13YZ=R;CHF14YZ=R;CHF15YZ=R;CHF20YZ=R;CHF25YZ=R;CHF30YZ=R;CHF40YZ=R;CHF50YZ=R</t>
-  </si>
-  <si>
     <t>CNYONZ=R;CNYTNZ=R;CNYSNZ=R;CNY1WZ=R;CNY2WZ=R;CNY1MZ=R;CNY2MZ=R;CNY3MZ=R;CNY6MZ=R;CNY9MZ=R;CNY1YZ=R;CNY1Y3MZ=R;CNY1Y6MZ=R;CNY1Y9MZ=R;CNY2YZ=R;CNY2Y3MZ=R;CNY2Y6MZ=R;CNY2Y9MZ=R;CNY3YZ=R;CNY3Y3MZ=R;CNY3Y6MZ=R;CNY3Y9MZ=R;CNY4YZ=R;CNY4Y3MZ=R;CNY4Y6MZ=R;CNY4Y9MZ=R;CNY5YZ=R;CNY5Y3MZ=R;CNY5Y6MZ=R;CNY5Y9MZ=R;CNY6YZ=R;CNY6Y3MZ=R;CNY6Y6MZ=R;CNY6Y9MZ=R;CNY7YZ=R;CNY7Y3MZ=R;CNY7Y6MZ=R;CNY7Y9MZ=R;CNY8YZ=R;CNY8Y3MZ=R;CNY8Y6MZ=R;CNY8Y9MZ=R;CNY9YZ=R;CNY9Y3MZ=R;CNY9Y6MZ=R;CNY9Y9MZ=R;CNY10YZ=R;CNY11YZ=R;CNY12YZ=R;CNY13YZ=R;CNY14YZ=R;CNY15YZ=R;CNY20YZ=R;CNY25YZ=R;CNY30YZ=R;CNY40YZ=R;CNY50YZ=R</t>
   </si>
   <si>
-    <t>CZKONZ=R;CZKTNZ=R;CZKSNZ=R;CZK1WZ=R;CZK2WZ=R;CZK1MZ=R;CZK2MZ=R;CZK3MZ=R;CZK6MZ=R;CZK9MZ=R;CZK1YZ=R;CZK1Y3MZ=R;CZK1Y6MZ=R;CZK1Y9MZ=R;CZK2YZ=R;CZK2Y3MZ=R;CZK2Y6MZ=R;CZK2Y9MZ=R;CZK3YZ=R;CZK3Y3MZ=R;CZK3Y6MZ=R;CZK3Y9MZ=R;CZK4YZ=R;CZK4Y3MZ=R;CZK4Y6MZ=R;CZK4Y9MZ=R;CZK5YZ=R;CZK5Y3MZ=R;CZK5Y6MZ=R;CZK5Y9MZ=R;CZK6YZ=R;CZK6Y3MZ=R;CZK6Y6MZ=R;CZK6Y9MZ=R;CZK7YZ=R;CZK7Y3MZ=R;CZK7Y6MZ=R;CZK7Y9MZ=R;CZK8YZ=R;CZK8Y3MZ=R;CZK8Y6MZ=R;CZK8Y9MZ=R;CZK9YZ=R;CZK9Y3MZ=R;CZK9Y6MZ=R;CZK9Y9MZ=R;CZK10YZ=R;CZK11YZ=R;CZK12YZ=R;CZK13YZ=R;CZK14YZ=R;CZK15YZ=R;CZK20YZ=R;CZK25YZ=R;CZK30YZ=R;CZK40YZ=R;CZK50YZ=R</t>
-  </si>
-  <si>
     <t>EURONZ=R;EURTNZ=R;EURSNZ=R;EUR1WZ=R;EUR2WZ=R;EUR1MZ=R;EUR2MZ=R;EUR3MZ=R;EUR6MZ=R;EUR9MZ=R;EUR1YZ=R;EUR1Y3MZ=R;EUR1Y6MZ=R;EUR1Y9MZ=R;EUR2YZ=R;EUR2Y3MZ=R;EUR2Y6MZ=R;EUR2Y9MZ=R;EUR3YZ=R;EUR3Y3MZ=R;EUR3Y6MZ=R;EUR3Y9MZ=R;EUR4YZ=R;EUR4Y3MZ=R;EUR4Y6MZ=R;EUR4Y9MZ=R;EUR5YZ=R;EUR5Y3MZ=R;EUR5Y6MZ=R;EUR5Y9MZ=R;EUR6YZ=R;EUR6Y3MZ=R;EUR6Y6MZ=R;EUR6Y9MZ=R;EUR7YZ=R;EUR7Y3MZ=R;EUR7Y6MZ=R;EUR7Y9MZ=R;EUR8YZ=R;EUR8Y3MZ=R;EUR8Y6MZ=R;EUR8Y9MZ=R;EUR9YZ=R;EUR9Y3MZ=R;EUR9Y6MZ=R;EUR9Y9MZ=R;EUR10YZ=R;EUR11YZ=R;EUR12YZ=R;EUR13YZ=R;EUR14YZ=R;EUR15YZ=R;EUR20YZ=R;EUR25YZ=R;EUR30YZ=R;EUR40YZ=R;EUR50YZ=R</t>
   </si>
   <si>
     <t>GBPONZ=R;GBPTNZ=R;GBPSNZ=R;GBP1WZ=R;GBP2WZ=R;GBP1MZ=R;GBP2MZ=R;GBP3MZ=R;GBP6MZ=R;GBP9MZ=R;GBP1YZ=R;GBP1Y3MZ=R;GBP1Y6MZ=R;GBP1Y9MZ=R;GBP2YZ=R;GBP2Y3MZ=R;GBP2Y6MZ=R;GBP2Y9MZ=R;GBP3YZ=R;GBP3Y3MZ=R;GBP3Y6MZ=R;GBP3Y9MZ=R;GBP4YZ=R;GBP4Y3MZ=R;GBP4Y6MZ=R;GBP4Y9MZ=R;GBP5YZ=R;GBP5Y3MZ=R;GBP5Y6MZ=R;GBP5Y9MZ=R;GBP6YZ=R;GBP6Y3MZ=R;GBP6Y6MZ=R;GBP6Y9MZ=R;GBP7YZ=R;GBP7Y3MZ=R;GBP7Y6MZ=R;GBP7Y9MZ=R;GBP8YZ=R;GBP8Y3MZ=R;GBP8Y6MZ=R;GBP8Y9MZ=R;GBP9YZ=R;GBP9Y3MZ=R;GBP9Y6MZ=R;GBP9Y9MZ=R;GBP10YZ=R;GBP11YZ=R;GBP12YZ=R;GBP13YZ=R;GBP14YZ=R;GBP15YZ=R;GBP20YZ=R;GBP25YZ=R;GBP30YZ=R;GBP40YZ=R;GBP50YZ=R</t>
   </si>
   <si>
-    <t>HKDONZ=R;HKDTNZ=R;HKDSNZ=R;HKD1WZ=R;HKD2WZ=R;HKD1MZ=R;HKD2MZ=R;HKD3MZ=R;HKD6MZ=R;HKD9MZ=R;HKD1YZ=R;HKD1Y3MZ=R;HKD1Y6MZ=R;HKD1Y9MZ=R;HKD2YZ=R;HKD2Y3MZ=R;HKD2Y6MZ=R;HKD2Y9MZ=R;HKD3YZ=R;HKD3Y3MZ=R;HKD3Y6MZ=R;HKD3Y9MZ=R;HKD4YZ=R;HKD4Y3MZ=R;HKD4Y6MZ=R;HKD4Y9MZ=R;HKD5YZ=R;HKD5Y3MZ=R;HKD5Y6MZ=R;HKD5Y9MZ=R;HKD6YZ=R;HKD6Y3MZ=R;HKD6Y6MZ=R;HKD6Y9MZ=R;HKD7YZ=R;HKD7Y3MZ=R;HKD7Y6MZ=R;HKD7Y9MZ=R;HKD8YZ=R;HKD8Y3MZ=R;HKD8Y6MZ=R;HKD8Y9MZ=R;HKD9YZ=R;HKD9Y3MZ=R;HKD9Y6MZ=R;HKD9Y9MZ=R;HKD10YZ=R;HKD11YZ=R;HKD12YZ=R;HKD13YZ=R;HKD14YZ=R;HKD15YZ=R;HKD20YZ=R;HKD25YZ=R;HKD30YZ=R;HKD40YZ=R;HKD50YZ=R</t>
-  </si>
-  <si>
-    <t>JPYONZ=R;JPYTNZ=R;JPYSNZ=R;JPY1WZ=R;JPY2WZ=R;JPY1MZ=R;JPY2MZ=R;JPY3MZ=R;JPY6MZ=R;JPY9MZ=R;JPY1YZ=R;JPY1Y3MZ=R;JPY1Y6MZ=R;JPY1Y9MZ=R;JPY2YZ=R;JPY2Y3MZ=R;JPY2Y6MZ=R;JPY2Y9MZ=R;JPY3YZ=R;JPY3Y3MZ=R;JPY3Y6MZ=R;JPY3Y9MZ=R;JPY4YZ=R;JPY4Y3MZ=R;JPY4Y6MZ=R;JPY4Y9MZ=R;JPY5YZ=R;JPY5Y3MZ=R;JPY5Y6MZ=R;JPY5Y9MZ=R;JPY6YZ=R;JPY6Y3MZ=R;JPY6Y6MZ=R;JPY6Y9MZ=R;JPY7YZ=R;JPY7Y3MZ=R;JPY7Y6MZ=R;JPY7Y9MZ=R;JPY8YZ=R;JPY8Y3MZ=R;JPY8Y6MZ=R;JPY8Y9MZ=R;JPY9YZ=R;JPY9Y3MZ=R;JPY9Y6MZ=R;JPY9Y9MZ=R;JPY10YZ=R;JPY11YZ=R;JPY12YZ=R;JPY13YZ=R;JPY14YZ=R;JPY15YZ=R;JPY20YZ=R;JPY25YZ=R;JPY30YZ=R;JPY40YZ=R;JPY50YZ=R</t>
-  </si>
-  <si>
-    <t>KRWONZ=R;KRWTNZ=R;KRWSNZ=R;KRW1WZ=R;KRW2WZ=R;KRW1MZ=R;KRW2MZ=R;KRW3MZ=R;KRW6MZ=R;KRW9MZ=R;KRW1YZ=R;KRW1Y3MZ=R;KRW1Y6MZ=R;KRW1Y9MZ=R;KRW2YZ=R;KRW2Y3MZ=R;KRW2Y6MZ=R;KRW2Y9MZ=R;KRW3YZ=R;KRW3Y3MZ=R;KRW3Y6MZ=R;KRW3Y9MZ=R;KRW4YZ=R;KRW4Y3MZ=R;KRW4Y6MZ=R;KRW4Y9MZ=R;KRW5YZ=R;KRW5Y3MZ=R;KRW5Y6MZ=R;KRW5Y9MZ=R;KRW6YZ=R;KRW6Y3MZ=R;KRW6Y6MZ=R;KRW6Y9MZ=R;KRW7YZ=R;KRW7Y3MZ=R;KRW7Y6MZ=R;KRW7Y9MZ=R;KRW8YZ=R;KRW8Y3MZ=R;KRW8Y6MZ=R;KRW8Y9MZ=R;KRW9YZ=R;KRW9Y3MZ=R;KRW9Y6MZ=R;KRW9Y9MZ=R;KRW10YZ=R;KRW11YZ=R;KRW12YZ=R;KRW13YZ=R;KRW14YZ=R;KRW15YZ=R;KRW20YZ=R;KRW25YZ=R;KRW30YZ=R;KRW40YZ=R;KRW50YZ=R</t>
-  </si>
-  <si>
-    <t>NOKONZ=R;NOKTNZ=R;NOKSNZ=R;NOK1WZ=R;NOK2WZ=R;NOK1MZ=R;NOK2MZ=R;NOK3MZ=R;NOK6MZ=R;NOK9MZ=R;NOK1YZ=R;NOK1Y3MZ=R;NOK1Y6MZ=R;NOK1Y9MZ=R;NOK2YZ=R;NOK2Y3MZ=R;NOK2Y6MZ=R;NOK2Y9MZ=R;NOK3YZ=R;NOK3Y3MZ=R;NOK3Y6MZ=R;NOK3Y9MZ=R;NOK4YZ=R;NOK4Y3MZ=R;NOK4Y6MZ=R;NOK4Y9MZ=R;NOK5YZ=R;NOK5Y3MZ=R;NOK5Y6MZ=R;NOK5Y9MZ=R;NOK6YZ=R;NOK6Y3MZ=R;NOK6Y6MZ=R;NOK6Y9MZ=R;NOK7YZ=R;NOK7Y3MZ=R;NOK7Y6MZ=R;NOK7Y9MZ=R;NOK8YZ=R;NOK8Y3MZ=R;NOK8Y6MZ=R;NOK8Y9MZ=R;NOK9YZ=R;NOK9Y3MZ=R;NOK9Y6MZ=R;NOK9Y9MZ=R;NOK10YZ=R;NOK11YZ=R;NOK12YZ=R;NOK13YZ=R;NOK14YZ=R;NOK15YZ=R;NOK20YZ=R;NOK25YZ=R;NOK30YZ=R;NOK40YZ=R;NOK50YZ=R</t>
-  </si>
-  <si>
-    <t>MXNONZ=R;MXNTNZ=R;MXNSNZ=R;MXN1WZ=R;MXN2WZ=R;MXN1MZ=R;MXN2MZ=R;MXN3MZ=R;MXN6MZ=R;MXN9MZ=R;MXN1YZ=R;MXN1Y3MZ=R;MXN1Y6MZ=R;MXN1Y9MZ=R;MXN2YZ=R;MXN2Y3MZ=R;MXN2Y6MZ=R;MXN2Y9MZ=R;MXN3YZ=R;MXN3Y3MZ=R;MXN3Y6MZ=R;MXN3Y9MZ=R;MXN4YZ=R;MXN4Y3MZ=R;MXN4Y6MZ=R;MXN4Y9MZ=R;MXN5YZ=R;MXN5Y3MZ=R;MXN5Y6MZ=R;MXN5Y9MZ=R;MXN6YZ=R;MXN6Y3MZ=R;MXN6Y6MZ=R;MXN6Y9MZ=R;MXN7YZ=R;MXN7Y3MZ=R;MXN7Y6MZ=R;MXN7Y9MZ=R;MXN8YZ=R;MXN8Y3MZ=R;MXN8Y6MZ=R;MXN8Y9MZ=R;MXN9YZ=R;MXN9Y3MZ=R;MXN9Y6MZ=R;MXN9Y9MZ=R;MXN10YZ=R;MXN11YZ=R;MXN12YZ=R;MXN13YZ=R;MXN14YZ=R;MXN15YZ=R;MXN20YZ=R;MXN25YZ=R;MXN30YZ=R;MXN40YZ=R;MXN50YZ=R</t>
-  </si>
-  <si>
-    <t>PENONZ=R;PENTNZ=R;PENSNZ=R;PEN1WZ=R;PEN2WZ=R;PEN1MZ=R;PEN2MZ=R;PEN3MZ=R;PEN6MZ=R;PEN9MZ=R;PEN1YZ=R;PEN1Y3MZ=R;PEN1Y6MZ=R;PEN1Y9MZ=R;PEN2YZ=R;PEN2Y3MZ=R;PEN2Y6MZ=R;PEN2Y9MZ=R;PEN3YZ=R;PEN3Y3MZ=R;PEN3Y6MZ=R;PEN3Y9MZ=R;PEN4YZ=R;PEN4Y3MZ=R;PEN4Y6MZ=R;PEN4Y9MZ=R;PEN5YZ=R;PEN5Y3MZ=R;PEN5Y6MZ=R;PEN5Y9MZ=R;PEN6YZ=R;PEN6Y3MZ=R;PEN6Y6MZ=R;PEN6Y9MZ=R;PEN7YZ=R;PEN7Y3MZ=R;PEN7Y6MZ=R;PEN7Y9MZ=R;PEN8YZ=R;PEN8Y3MZ=R;PEN8Y6MZ=R;PEN8Y9MZ=R;PEN9YZ=R;PEN9Y3MZ=R;PEN9Y6MZ=R;PEN9Y9MZ=R;PEN10YZ=R;PEN11YZ=R;PEN12YZ=R;PEN13YZ=R;PEN14YZ=R;PEN15YZ=R;PEN20YZ=R;PEN25YZ=R;PEN30YZ=R;PEN40YZ=R;PEN50YZ=R</t>
-  </si>
-  <si>
-    <t>PLNONZ=R;PLNTNZ=R;PLNSNZ=R;PLN1WZ=R;PLN2WZ=R;PLN1MZ=R;PLN2MZ=R;PLN3MZ=R;PLN6MZ=R;PLN9MZ=R;PLN1YZ=R;PLN1Y3MZ=R;PLN1Y6MZ=R;PLN1Y9MZ=R;PLN2YZ=R;PLN2Y3MZ=R;PLN2Y6MZ=R;PLN2Y9MZ=R;PLN3YZ=R;PLN3Y3MZ=R;PLN3Y6MZ=R;PLN3Y9MZ=R;PLN4YZ=R;PLN4Y3MZ=R;PLN4Y6MZ=R;PLN4Y9MZ=R;PLN5YZ=R;PLN5Y3MZ=R;PLN5Y6MZ=R;PLN5Y9MZ=R;PLN6YZ=R;PLN6Y3MZ=R;PLN6Y6MZ=R;PLN6Y9MZ=R;PLN7YZ=R;PLN7Y3MZ=R;PLN7Y6MZ=R;PLN7Y9MZ=R;PLN8YZ=R;PLN8Y3MZ=R;PLN8Y6MZ=R;PLN8Y9MZ=R;PLN9YZ=R;PLN9Y3MZ=R;PLN9Y6MZ=R;PLN9Y9MZ=R;PLN10YZ=R;PLN11YZ=R;PLN12YZ=R;PLN13YZ=R;PLN14YZ=R;PLN15YZ=R;PLN20YZ=R;PLN25YZ=R;PLN30YZ=R;PLN40YZ=R;PLN50YZ=R</t>
-  </si>
-  <si>
-    <t>RUBONZ=R;RUBTNZ=R;RUBSNZ=R;RUB1WZ=R;RUB2WZ=R;RUB1MZ=R;RUB2MZ=R;RUB3MZ=R;RUB6MZ=R;RUB9MZ=R;RUB1YZ=R;RUB1Y3MZ=R;RUB1Y6MZ=R;RUB1Y9MZ=R;RUB2YZ=R;RUB2Y3MZ=R;RUB2Y6MZ=R;RUB2Y9MZ=R;RUB3YZ=R;RUB3Y3MZ=R;RUB3Y6MZ=R;RUB3Y9MZ=R;RUB4YZ=R;RUB4Y3MZ=R;RUB4Y6MZ=R;RUB4Y9MZ=R;RUB5YZ=R;RUB5Y3MZ=R;RUB5Y6MZ=R;RUB5Y9MZ=R;RUB6YZ=R;RUB6Y3MZ=R;RUB6Y6MZ=R;RUB6Y9MZ=R;RUB7YZ=R;RUB7Y3MZ=R;RUB7Y6MZ=R;RUB7Y9MZ=R;RUB8YZ=R;RUB8Y3MZ=R;RUB8Y6MZ=R;RUB8Y9MZ=R;RUB9YZ=R;RUB9Y3MZ=R;RUB9Y6MZ=R;RUB9Y9MZ=R;RUB10YZ=R;RUB11YZ=R;RUB12YZ=R;RUB13YZ=R;RUB14YZ=R;RUB15YZ=R;RUB20YZ=R;RUB25YZ=R;RUB30YZ=R;RUB40YZ=R;RUB50YZ=R</t>
-  </si>
-  <si>
     <t>SEKONZ=R;SEKTNZ=R;SEKSNZ=R;SEK1WZ=R;SEK2WZ=R;SEK1MZ=R;SEK2MZ=R;SEK3MZ=R;SEK6MZ=R;SEK9MZ=R;SEK1YZ=R;SEK1Y3MZ=R;SEK1Y6MZ=R;SEK1Y9MZ=R;SEK2YZ=R;SEK2Y3MZ=R;SEK2Y6MZ=R;SEK2Y9MZ=R;SEK3YZ=R;SEK3Y3MZ=R;SEK3Y6MZ=R;SEK3Y9MZ=R;SEK4YZ=R;SEK4Y3MZ=R;SEK4Y6MZ=R;SEK4Y9MZ=R;SEK5YZ=R;SEK5Y3MZ=R;SEK5Y6MZ=R;SEK5Y9MZ=R;SEK6YZ=R;SEK6Y3MZ=R;SEK6Y6MZ=R;SEK6Y9MZ=R;SEK7YZ=R;SEK7Y3MZ=R;SEK7Y6MZ=R;SEK7Y9MZ=R;SEK8YZ=R;SEK8Y3MZ=R;SEK8Y6MZ=R;SEK8Y9MZ=R;SEK9YZ=R;SEK9Y3MZ=R;SEK9Y6MZ=R;SEK9Y9MZ=R;SEK10YZ=R;SEK11YZ=R;SEK12YZ=R;SEK13YZ=R;SEK14YZ=R;SEK15YZ=R;SEK20YZ=R;SEK25YZ=R;SEK30YZ=R;SEK40YZ=R;SEK50YZ=R</t>
   </si>
   <si>
-    <t>SGDONZ=R;SGDTNZ=R;SGDSNZ=R;SGD1WZ=R;SGD2WZ=R;SGD1MZ=R;SGD2MZ=R;SGD3MZ=R;SGD6MZ=R;SGD9MZ=R;SGD1YZ=R;SGD1Y3MZ=R;SGD1Y6MZ=R;SGD1Y9MZ=R;SGD2YZ=R;SGD2Y3MZ=R;SGD2Y6MZ=R;SGD2Y9MZ=R;SGD3YZ=R;SGD3Y3MZ=R;SGD3Y6MZ=R;SGD3Y9MZ=R;SGD4YZ=R;SGD4Y3MZ=R;SGD4Y6MZ=R;SGD4Y9MZ=R;SGD5YZ=R;SGD5Y3MZ=R;SGD5Y6MZ=R;SGD5Y9MZ=R;SGD6YZ=R;SGD6Y3MZ=R;SGD6Y6MZ=R;SGD6Y9MZ=R;SGD7YZ=R;SGD7Y3MZ=R;SGD7Y6MZ=R;SGD7Y9MZ=R;SGD8YZ=R;SGD8Y3MZ=R;SGD8Y6MZ=R;SGD8Y9MZ=R;SGD9YZ=R;SGD9Y3MZ=R;SGD9Y6MZ=R;SGD9Y9MZ=R;SGD10YZ=R;SGD11YZ=R;SGD12YZ=R;SGD13YZ=R;SGD14YZ=R;SGD15YZ=R;SGD20YZ=R;SGD25YZ=R;SGD30YZ=R;SGD40YZ=R;SGD50YZ=R</t>
-  </si>
-  <si>
-    <t>THBONZ=R;THBTNZ=R;THBSNZ=R;THB1WZ=R;THB2WZ=R;THB1MZ=R;THB2MZ=R;THB3MZ=R;THB6MZ=R;THB9MZ=R;THB1YZ=R;THB1Y3MZ=R;THB1Y6MZ=R;THB1Y9MZ=R;THB2YZ=R;THB2Y3MZ=R;THB2Y6MZ=R;THB2Y9MZ=R;THB3YZ=R;THB3Y3MZ=R;THB3Y6MZ=R;THB3Y9MZ=R;THB4YZ=R;THB4Y3MZ=R;THB4Y6MZ=R;THB4Y9MZ=R;THB5YZ=R;THB5Y3MZ=R;THB5Y6MZ=R;THB5Y9MZ=R;THB6YZ=R;THB6Y3MZ=R;THB6Y6MZ=R;THB6Y9MZ=R;THB7YZ=R;THB7Y3MZ=R;THB7Y6MZ=R;THB7Y9MZ=R;THB8YZ=R;THB8Y3MZ=R;THB8Y6MZ=R;THB8Y9MZ=R;THB9YZ=R;THB9Y3MZ=R;THB9Y6MZ=R;THB9Y9MZ=R;THB10YZ=R;THB11YZ=R;THB12YZ=R;THB13YZ=R;THB14YZ=R;THB15YZ=R;THB20YZ=R;THB25YZ=R;THB30YZ=R;THB40YZ=R;THB50YZ=R</t>
-  </si>
-  <si>
     <t>ZARONZ=R;ZARTNZ=R;ZARSNZ=R;ZAR1WZ=R;ZAR2WZ=R;ZAR1MZ=R;ZAR2MZ=R;ZAR3MZ=R;ZAR6MZ=R;ZAR9MZ=R;ZAR1YZ=R;ZAR1Y3MZ=R;ZAR1Y6MZ=R;ZAR1Y9MZ=R;ZAR2YZ=R;ZAR2Y3MZ=R;ZAR2Y6MZ=R;ZAR2Y9MZ=R;ZAR3YZ=R;ZAR3Y3MZ=R;ZAR3Y6MZ=R;ZAR3Y9MZ=R;ZAR4YZ=R;ZAR4Y3MZ=R;ZAR4Y6MZ=R;ZAR4Y9MZ=R;ZAR5YZ=R;ZAR5Y3MZ=R;ZAR5Y6MZ=R;ZAR5Y9MZ=R;ZAR6YZ=R;ZAR6Y3MZ=R;ZAR6Y6MZ=R;ZAR6Y9MZ=R;ZAR7YZ=R;ZAR7Y3MZ=R;ZAR7Y6MZ=R;ZAR7Y9MZ=R;ZAR8YZ=R;ZAR8Y3MZ=R;ZAR8Y6MZ=R;ZAR8Y9MZ=R;ZAR9YZ=R;ZAR9Y3MZ=R;ZAR9Y6MZ=R;ZAR9Y9MZ=R;ZAR10YZ=R;ZAR11YZ=R;ZAR12YZ=R;ZAR13YZ=R;ZAR14YZ=R;ZAR15YZ=R;ZAR20YZ=R;ZAR25YZ=R;ZAR30YZ=R;ZAR40YZ=R;ZAR50YZ=R</t>
   </si>
   <si>
     <t>INROISONZ=R;INROISTNZ=R;INROISSNZ=R;INROIS1WZ=R;INROIS2WZ=R;INROIS1MZ=R;INROIS2MZ=R;INROIS3MZ=R;INROIS6MZ=R;INROIS9MZ=R;INROIS1YZ=R;INROIS1Y3MZ=R;INROIS1Y6MZ=R;INROIS1Y9MZ=R;INROIS2YZ=R;INROIS2Y3MZ=R;INROIS2Y6MZ=R;INROIS2Y9MZ=R;INROIS3YZ=R;INROIS3Y3MZ=R;INROIS3Y6MZ=R;INROIS3Y9MZ=R;INROIS4YZ=R;INROIS4Y3MZ=R;INROIS4Y6MZ=R;INROIS4Y9MZ=R;INROIS5YZ=R;INROIS5Y3MZ=R;INROIS5Y6MZ=R;INROIS5Y9MZ=R;INROIS6YZ=R;INROIS6Y3MZ=R;INROIS6Y6MZ=R;INROIS6Y9MZ=R;INROIS7YZ=R;INROIS7Y3MZ=R;INROIS7Y6MZ=R;INROIS7Y9MZ=R;INROIS8YZ=R;INROIS8Y3MZ=R;INROIS8Y6MZ=R;INROIS8Y9MZ=R;INROIS9YZ=R;INROIS9Y3MZ=R;INROIS9Y6MZ=R;INROIS9Y9MZ=R;INROIS10YZ=R;INROIS11YZ=R;INROIS12YZ=R;INROIS13YZ=R;INROIS14YZ=R;INROIS15YZ=R;INROIS20YZ=R;INROIS25YZ=R;INROIS30YZ=R;INROIS40YZ=R;INROIS50YZ=R</t>
-  </si>
-  <si>
-    <t>CLPOISONZ=R;CLPOISTNZ=R;CLPOISSNZ=R;CLPOIS1WZ=R;CLPOIS2WZ=R;CLPOIS1MZ=R;CLPOIS2MZ=R;CLPOIS3MZ=R;CLPOIS6MZ=R;CLPOIS9MZ=R;CLPOIS1YZ=R;CLPOIS1Y3MZ=R;CLPOIS1Y6MZ=R;CLPOIS1Y9MZ=R;CLPOIS2YZ=R;CLPOIS2Y3MZ=R;CLPOIS2Y6MZ=R;CLPOIS2Y9MZ=R;CLPOIS3YZ=R;CLPOIS3Y3MZ=R;CLPOIS3Y6MZ=R;CLPOIS3Y9MZ=R;CLPOIS4YZ=R;CLPOIS4Y3MZ=R;CLPOIS4Y6MZ=R;CLPOIS4Y9MZ=R;CLPOIS5YZ=R;CLPOIS5Y3MZ=R;CLPOIS5Y6MZ=R;CLPOIS5Y9MZ=R;CLPOIS6YZ=R;CLPOIS6Y3MZ=R;CLPOIS6Y6MZ=R;CLPOIS6Y9MZ=R;CLPOIS7YZ=R;CLPOIS7Y3MZ=R;CLPOIS7Y6MZ=R;CLPOIS7Y9MZ=R;CLPOIS8YZ=R;CLPOIS8Y3MZ=R;CLPOIS8Y6MZ=R;CLPOIS8Y9MZ=R;CLPOIS9YZ=R;CLPOIS9Y3MZ=R;CLPOIS9Y6MZ=R;CLPOIS9Y9MZ=R;CLPOIS10YZ=R;CLPOIS11YZ=R;CLPOIS12YZ=R;CLPOIS13YZ=R;CLPOIS14YZ=R;CLPOIS15YZ=R;CLPOIS20YZ=R;CLPOIS25YZ=R;CLPOIS30YZ=R;CLPOIS40YZ=R;CLPOIS50YZ=R</t>
-  </si>
-  <si>
-    <t>DKKONZ=R;DKKTNZ=R;DKKSNZ=R;DKK1WZ=R;DKK2WZ=R;DKK1MZ=R;DKK2MZ=R;DKK3MZ=R;DKK6MZ=R;DKK9MZ=R;DKK1YZ=R;DKK1Y3MZ=R;DKK1Y6MZ=R;DKK1Y9MZ=R;DKK2YZ=R;DKK2Y3MZ=R;DKK2Y6MZ=R;DKK2Y9MZ=R;DKK3YZ=R;DKK3Y3MZ=R;DKK3Y6MZ=R;DKK3Y9MZ=R;DKK4YZ=R;DKK4Y3MZ=R;DKK4Y6MZ=R;DKK4Y9MZ=R;DKK5YZ=R;DKK5Y3MZ=R;DKK5Y6MZ=R;DKK5Y9MZ=R;DKK6YZ=R;DKK6Y3MZ=R;DKK6Y6MZ=R;DKK6Y9MZ=R;DKK7YZ=R;DKK7Y3MZ=R;DKK7Y6MZ=R;DKK7Y9MZ=R;DKK8YZ=R;DKK8Y3MZ=R;DKK8Y6MZ=R;DKK8Y9MZ=R;DKK9YZ=R;DKK9Y3MZ=R;DKK9Y6MZ=R;DKK9Y9MZ=R;DKK10YZ=R;DKK11YZ=R;DKK12YZ=R;DKK13YZ=R;DKK14YZ=R;DKK15YZ=R;DKK20YZ=R;DKK25YZ=R;DKK30YZ=R;DKK40YZ=R;DKK50YZ=R</t>
   </si>
   <si>
     <t>AUD=;BGN=;BWP=;CAD=;CHF=;CLP=;CNY=;CZK=;DKK=;EUR=;GBP=;HKD=;INR=;JPY=;KRW=;MXN=;NOK=;PEN=;PLN=;RUB=;SEK=;SGD=;THB=;ZAR=</t>
@@ -431,12 +383,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -466,7 +418,7 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
@@ -476,95 +428,16 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>